<commit_message>
tratamento pra limite de nodes do graphql
</commit_message>
<xml_diff>
--- a/communitySmellsDataset.xlsx
+++ b/communitySmellsDataset.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O181"/>
+  <dimension ref="A1:O189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14000,6 +14000,606 @@
         </is>
       </c>
     </row>
+    <row r="182">
+      <c r="A182" s="2" t="n">
+        <v>181</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>https://github.com/altair-graphql/altair</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>altair</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>altair-graphql</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>03/25/2017</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N182" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="n">
+        <v>182</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>https://github.com/JabRef/jabref</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>jabref</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>JabRef</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>10/14/2003</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N183" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="n">
+        <v>183</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>https://github.com/pyladies/pyladies</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>pyladies</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>pyladies</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>04/19/2011</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N184" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="n">
+        <v>184</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>https://github.com/okfn-brasil/querido-diario</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>querido-diario</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>okfn-brasil</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>04/01/2018</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N185" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="n">
+        <v>185</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>https://github.com/pyladies/pyladies</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>pyladies</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>pyladies</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>04/19/2011</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N186" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="n">
+        <v>186</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>https://github.com/facebook/create-react-app</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>create-react-app</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>facebook</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>07/18/2016</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N187" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="n">
+        <v>187</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>https://github.com/JabRef/jabref</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>jabref</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>JabRef</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>10/14/2003</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N188" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="n">
+        <v>188</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>https://github.com/vuejs/core</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>vuejs</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>09/19/2018</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N189" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>